<commit_message>
research: Teams Counted column beside clubs in master + province workbooks
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/research/provinces/SportsHub-Alberta.xlsx
+++ b/docs/research/provinces/SportsHub-Alberta.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Club Sizes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Clubs'!$A$1:$P$204</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Clubs'!$A$1:$Q$204</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Leagues'!$A$1:$L$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Club-League Map'!$A$1:$E$240</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Contacts'!$A$1:$F$177</definedName>
@@ -65,11 +65,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P204"/>
+  <dimension ref="A1:Q204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -454,6 +455,7 @@
     <col width="11" customWidth="1" min="14" max="14"/>
     <col width="30" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -537,6 +539,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>Teams Counted</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -671,6 +678,9 @@
           <t>https://airdriebasketball.ca/executive</t>
         </is>
       </c>
+      <c r="Q3" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -959,6 +969,9 @@
           <t>Phone as reported in search result for byba.ca</t>
         </is>
       </c>
+      <c r="Q7" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1242,6 +1255,9 @@
           <t>Being replaced (with SoCal) by the new South Stoney Basketball Association CMBA zone as of 2026.</t>
         </is>
       </c>
+      <c r="Q11" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1659,6 +1675,9 @@
           <t>ABA member club; Nick Tancon — Director Boys Basketball; Mark Hogan lead coach</t>
         </is>
       </c>
+      <c r="Q17" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2138,6 +2157,9 @@
           <t>Former domain calgaryselects.ca now parked/expired — club status worth confirming</t>
         </is>
       </c>
+      <c r="Q24" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2617,6 +2639,9 @@
           <t>Community association (CMBA zone, NE Calgary, ages 6-17). Platform: RAMP InterActive (site + RAMP Registration Solutions). Full board on /executive: VP/Gym Coord Gary Dormer (gary.dormer@gmail.com), Treasurer Charlene Proulx (heycharlene@live.com), Secretary Liezel Erskine, Registrar Manpreet Jhinjar, Equipment Edyta Borges, Directors Eugene Danquah &amp; Sarah La Riviere — board uses personal emails, no org domain emails. ZoomInfo lists phone (403) 815-8056 and postal T3J 2R7 (unverified elsewhere, not put in phone field). Site TLS cert broken (fetched via proxy). Sources: http://eastprobasketball.ca/executive ; http://eastprobasketball.ca/ ; https://www.cmba.ab.ca/content/board-executive-and-committees ; https://www.zoominfo.com/c/east-pro-basketball/481522487</t>
         </is>
       </c>
+      <c r="Q31" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2858,6 +2883,9 @@
           <t>Site has 'Meet our President' page but name is JS-rendered and was not captured. | Also listed as: Excel Basketball Academy | enriched 2026-07-18</t>
         </is>
       </c>
+      <c r="Q34" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2992,6 +3020,9 @@
           <t>Also listed as: Far East Basketball Training League</t>
         </is>
       </c>
+      <c r="Q36" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3146,6 +3177,9 @@
           <t>ABA member listing 'Genesis Basketball'; Edmonton teams appear in EYBA/YP portals as Genesis YEG | enriched 2026-07-18</t>
         </is>
       </c>
+      <c r="Q38" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3461,6 +3495,9 @@
           <t>Also listed as: MENA Basketball Foundation</t>
         </is>
       </c>
+      <c r="Q43" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3724,6 +3761,9 @@
           <t>https://www.aybc.ca/2020-club-members-1/nw-warriors</t>
         </is>
       </c>
+      <c r="Q47" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3766,6 +3806,9 @@
           <t>Listed as 'No Limit Elite / Calgary' on ABA 2022-23 members list; no website found.</t>
         </is>
       </c>
+      <c r="Q48" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3905,6 +3948,9 @@
           <t>Also branded 'NW Calgary Basketball Club'; Calgary Surge youth partner</t>
         </is>
       </c>
+      <c r="Q50" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3967,6 +4013,9 @@
           <t>https://www.aybc.ca/2020-club-members-1/purehoops-basketball-club</t>
         </is>
       </c>
+      <c r="Q51" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4225,6 +4274,9 @@
           <t>'Rise Up Hoops / Calgary' on ABA 2022-23 member list; multiple brand names map to one operation.</t>
         </is>
       </c>
+      <c r="Q55" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4359,6 +4411,9 @@
           <t>States member in good standing with Alberta Basketball</t>
         </is>
       </c>
+      <c r="Q57" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4833,6 +4888,9 @@
           <t>Canada Basketball verified; Jr. NBA partnership</t>
         </is>
       </c>
+      <c r="Q64" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5260,6 +5318,9 @@
           <t>ABA member club listing</t>
         </is>
       </c>
+      <c r="Q70" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -6332,6 +6393,9 @@
           <t>https://www.cochraneminorbasketball.com</t>
         </is>
       </c>
+      <c r="Q86" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6657,6 +6721,9 @@
           <t>enriched 2026-07-18</t>
         </is>
       </c>
+      <c r="Q91" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -6801,6 +6868,9 @@
           <t>Nonprofit, ~5 years old, development-first philosophy</t>
         </is>
       </c>
+      <c r="Q93" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -7280,6 +7350,9 @@
           <t>Canada Basketball &amp; Alberta Basketball Verified Club; second phone (780) 903-7455 | enriched 2026-07-18</t>
         </is>
       </c>
+      <c r="Q100" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -7357,6 +7430,9 @@
           <t>Edmonton branch of Genesis Basketball (Calgary org genesisbasketball.net); 'Genesis Basketball' on PSO member registry</t>
         </is>
       </c>
+      <c r="Q101" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -7841,6 +7917,9 @@
           <t>Type: community association — NE Edmonton zone of Edmonton Youth Basketball (EYBA), ages 5-17. Full executive on http://northeastbasketball.com/executive: Donna Haggstrom (Executive Director, info@), Robin Bussiere (President &amp; Coach Liaison, CoachLiaison@northeastbasketball.com), Peter Piekema (Treasurer), Jasmine Murphy (Secretary), Rebecca VandenBorn (Registrar). PLATFORM INTEL: RAMP InterActive (website + registration + RAMP Team App). Site cert broken on HTTPS — use http.</t>
         </is>
       </c>
+      <c r="Q108" t="n">
+        <v>37</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -7960,6 +8039,9 @@
           <t>Facebook-only web presence; EYBA registered club member | Also listed as: Northern Hoops Selects</t>
         </is>
       </c>
+      <c r="Q110" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -8084,6 +8166,9 @@
           <t>Type: community association — formed 2012 by merger of Wellington, Aldergrove, Willowby, Parkview and Glenora community programs (NW Edmonton zone). Executive on http://northwestbasketball.ca/executive: Carr Miceli (President, info@), Brad Coleman (VP), Anne-Marie Vaasjo (Treasurer, treasurer@northwestbasketball.ca), Remko Oosterhuis (Registration Director), Rheann Kelly (Secretary/Social Media). PLATFORM INTEL: RAMP InterActive (website + registration). Site cert broken on HTTPS — use http. | Also listed as: Northwest Zone Basketball Association</t>
         </is>
       </c>
+      <c r="Q112" t="n">
+        <v>59</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -8156,6 +8241,9 @@
           <t>Partners with Alberta Basketball | enriched 2026-07-18</t>
         </is>
       </c>
+      <c r="Q113" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -8208,6 +8296,9 @@
           <t>EYBA clubs page links 'Rockets Basketball' to rocketsbasketball.ca which resolves to a Cole Harbour NS club — link appears stale/wrong; Edmonton club identity unverified beyond EYBA team pages</t>
         </is>
       </c>
+      <c r="Q114" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -8260,6 +8351,9 @@
           <t>EYBA clubs page links this member to rocketsbasketball.ca, which is actually a Cole Harbour, Nova Scotia association — stale/wrong link; Edmonton Rockets' own web presence not found</t>
         </is>
       </c>
+      <c r="Q115" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -8419,6 +8513,9 @@
           <t>One of four Edmonton quadrant zone associations under EYBA | Also listed as: Southwest Basketball Association</t>
         </is>
       </c>
+      <c r="Q117" t="n">
+        <v>66</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -8501,6 +8598,9 @@
           <t>Incorporated June 2026; tournament operator at scale (400+ teams projected) — both a club and an events business | Type: private club/academy, founded January 2011 by Ron Hopkins; site notes 'Swoosh Canada Basketball Inc.' officially incorporated June 2026. Phone/email route directly to Hopkins. Custom website (not RAMP/TeamLinkt/SportsEngine). Sources: https://www.swooshcanada.com/ (address) ; https://www.swooshcanada.com/contact-us (phone/email) ; https://www.swooshcanada.com/our-story (founder)</t>
         </is>
       </c>
+      <c r="Q118" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -8722,6 +8822,9 @@
           <t>enriched 2026-07-18</t>
         </is>
       </c>
+      <c r="Q121" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -9868,6 +9971,9 @@
           <t>Type: community association / rep club, non-profit; plays in EYBA. Site hosted on RAMP InterActive. Address is a PO box (no street address or phone published). Executive at https://www.leduclightning.com/executive: President Chris Burke (president@leduclightning.com), VP Kelli Warren, Secretary Randi Stassen, Treasurer Jaimie Delwisch, Registrar Kelly Valentine (registrar@leduclightning.com), EYBA Director Erin Kivitt. Sources: https://www.leduclightning.com/ ; https://www.leduclightning.com/executive</t>
         </is>
       </c>
+      <c r="Q139" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -10193,6 +10299,9 @@
           <t>Self-described as southern Alberta's only ABA-sanctioned organization; on ABA member list as 'LMBA'. Second email lethbridgeminorbasketball@gmail.com. Club-team brand 'Lethbridge Express (LMBA)' pinned separately on ABA club map.</t>
         </is>
       </c>
+      <c r="Q144" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -11277,6 +11386,9 @@
           <t>Also uses morinvilleyouthbasketball@gmail.com</t>
         </is>
       </c>
+      <c r="Q161" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -11493,6 +11605,9 @@
           <t>Record 2025-26 season per Western Wheel local news (westernwheel.ca). | Also listed as: Okotoks Basketball Association (OBA)</t>
         </is>
       </c>
+      <c r="Q164" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -11994,6 +12109,9 @@
           <t>Appears on Alberta Basketball association/club listing; Raymond is one of Alberta's most storied basketball towns (Raymond Comets HS dynasty) but no standalone youth-club web presence found.</t>
         </is>
       </c>
+      <c r="Q172" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -13111,6 +13229,9 @@
           <t>Street address/phone from Yelp/ZoomInfo listings; email is from official site</t>
         </is>
       </c>
+      <c r="Q188" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -13272,6 +13393,9 @@
           <t>http://www.parklandbasketball.ca/</t>
         </is>
       </c>
+      <c r="Q191" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -13344,6 +13468,9 @@
           <t>Do not confuse with parklandbasketball.com (US club) | Type: community league + rep program (Parkland Pride) serving Spruce Grove, Stony Plain, Parkland County; member of EYBA (Edmonton Youth Basketball Association). Site hosted on RAMP InterActive; registration via parklandpride.rampregistrations.com. Executives at http://www.parklandbasketball.ca/executive: President Jason Hackman (jasonh@parklandbasketball.ca), VP/Program Director Jay Ouellette (vicepresident@parklandbasketball.ca), Treasurer Jocelyn Couture, Secretary/Registrar Julie Ouellette (administration@parklandbasketball.ca), Past President Robert Bull. Secondary site/email: parklandbasketball.wordpress.com / parklandbasketball@gmail.com. Footer shows only 'Spruce Grove, AB' — no street address or phone published. Sources: http://www.parklandbasketball.ca/executive ; https://parklandbasketball.wordpress.com/about/</t>
         </is>
       </c>
+      <c r="Q192" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -13478,6 +13605,9 @@
           <t>Distinct from SAYBL (separate St. Albert house-league org) | Type: community rep/development club (since 2001). Site hosted on RAMP InterActive. Full executive board published at https://www.stalbertslam.com/executive — President Tanner Wilson (President@stalbertslam.com), VP Abdelrahman Elsabbagh (VP@stalbertslam.com), Secretary Rick Walters, Treasurer Katy Illner, Registrar Denise Barrett (Registrations@stalbertslam.com). No street address or phone published anywhere on site (contact page https://www.stalbertslam.com/content/contact-us is email-only). Socials: instagram.com/st.albertslam. Sources: https://www.stalbertslam.com/executive ; https://www.stalbertslam.com/content/contact-us</t>
         </is>
       </c>
+      <c r="Q194" t="n">
+        <v>42</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -13617,6 +13747,9 @@
           <t>Competitive-intel: one of the few Edmonton-region orgs on SportsEngine rather than RAMP | Type: community house league (boys &amp; girls ages 8-15), volunteer non-profit. Site hosted on SportsEngine (mirror: saybl.sportngin.com). Board published at https://www.saybl.ca/board: President/Treasurer Alana Gregson, VP Angela Lippolt, Secretary Jen Berglind, plus ~11 directors (registration Kayla/Ryan Groten, communications Jon/Laurie Fitzlaff, coach coordinator Sarah Dukovac). SportsEngine org directory lists board member Antony Bernadou as org contact and address only as 'St. Albert, AB T8N 0A1' (no street). saybl.ca blocks bots (403) — data pulled via direct HTML fetch. Sources: https://www.saybl.ca/board ; https://www.sportsengine.com/org/st-albert-youth-basketball-league</t>
         </is>
       </c>
+      <c r="Q196" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -13999,6 +14132,9 @@
           <t>On ABA 2022/23 good standing and official club map.</t>
         </is>
       </c>
+      <c r="Q202" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -14135,7 +14271,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P204"/>
+  <autoFilter ref="A1:Q204"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
research: Bow River corrected 89→74 — independent verification (owner challenge)
Second agent enumerated Bow River's own calendar API across all 8 CMBA
divisions: 74 unique teams, gap-free numbering (U18 Girls = 0). Original
league-API unique-name count overshot ~20%. Corrected in raw data, Club
Sizes tabs, Teams Counted column. All counts remain labeled directional.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/research/provinces/SportsHub-Alberta.xlsx
+++ b/docs/research/provinces/SportsHub-Alberta.xlsx
@@ -26257,11 +26257,11 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>89</v>
+        <v>74</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>CMBA Fall/Winter League (Calgary Minor=89</t>
+          <t>CMBA Fall/Winter=74 (verified 2026-07-18)</t>
         </is>
       </c>
     </row>

</xml_diff>